<commit_message>
Tickets: add protocol-attendance column L and deviation metric
Set column L in «Реализованные билеты» to «Посещаемость по протоколу» and
default it to 0 for every match row (the club fills real protocol figures
later). Add two metrics to «Расчеты» in the previously-blank rows 17 and 20
(so no existing cell references shift): protocol attendance for the season,
and «Отклонение от протокола» = protocol attendance / total tickets. Both are
formulas over column L, recalculating as L is filled in.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/tickets_calc.xlsx
+++ b/output/tickets_calc.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="L2" s="44" t="inlineStr">
         <is>
-          <t>Комментарий</t>
+          <t>Посещаемость по протоколу</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,9 @@
         <f>SUM(C5:J5)</f>
         <v/>
       </c>
-      <c r="L5" s="10" t="n"/>
+      <c r="L5" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M5" s="11" t="n"/>
     </row>
     <row r="6">
@@ -1259,7 +1261,9 @@
         <f>SUM(C6:J6)</f>
         <v/>
       </c>
-      <c r="L6" s="10" t="n"/>
+      <c r="L6" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M6" s="11" t="n"/>
     </row>
     <row r="7" ht="15.95" customHeight="1" s="48">
@@ -1297,7 +1301,9 @@
         <f>SUM(C7:J7)</f>
         <v/>
       </c>
-      <c r="L7" s="10" t="n"/>
+      <c r="L7" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M7" s="11" t="n"/>
     </row>
     <row r="8">
@@ -1335,7 +1341,9 @@
         <f>SUM(C8:J8)</f>
         <v/>
       </c>
-      <c r="L8" s="10" t="n"/>
+      <c r="L8" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M8" s="11" t="n"/>
     </row>
     <row r="9" ht="15.95" customHeight="1" s="48">
@@ -1373,7 +1381,9 @@
         <f>SUM(C9:J9)</f>
         <v/>
       </c>
-      <c r="L9" s="10" t="n"/>
+      <c r="L9" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M9" s="11" t="n"/>
     </row>
     <row r="10">
@@ -1411,7 +1421,9 @@
         <f>SUM(C10:J10)</f>
         <v/>
       </c>
-      <c r="L10" s="10" t="n"/>
+      <c r="L10" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M10" s="11" t="n"/>
     </row>
     <row r="11" ht="15.95" customHeight="1" s="48">
@@ -1449,7 +1461,9 @@
         <f>SUM(C11:J11)</f>
         <v/>
       </c>
-      <c r="L11" s="10" t="n"/>
+      <c r="L11" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M11" s="11" t="n"/>
     </row>
     <row r="12">
@@ -1487,7 +1501,9 @@
         <f>SUM(C12:J12)</f>
         <v/>
       </c>
-      <c r="L12" s="10" t="n"/>
+      <c r="L12" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M12" s="11" t="n"/>
     </row>
     <row r="13" ht="15.95" customHeight="1" s="48">
@@ -1525,7 +1541,9 @@
         <f>SUM(C13:J13)</f>
         <v/>
       </c>
-      <c r="L13" s="10" t="n"/>
+      <c r="L13" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M13" s="11" t="n"/>
     </row>
     <row r="14">
@@ -1563,7 +1581,9 @@
         <f>SUM(C14:J14)</f>
         <v/>
       </c>
-      <c r="L14" s="10" t="n"/>
+      <c r="L14" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M14" s="11" t="n"/>
     </row>
     <row r="15" ht="15.95" customHeight="1" s="48">
@@ -1601,7 +1621,9 @@
         <f>SUM(C15:J15)</f>
         <v/>
       </c>
-      <c r="L15" s="10" t="n"/>
+      <c r="L15" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M15" s="11" t="n"/>
     </row>
     <row r="16">
@@ -1639,7 +1661,9 @@
         <f>SUM(C16:J16)</f>
         <v/>
       </c>
-      <c r="L16" s="10" t="n"/>
+      <c r="L16" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M16" s="11" t="n"/>
     </row>
     <row r="17" ht="15.95" customHeight="1" s="48">
@@ -1677,7 +1701,9 @@
         <f>SUM(C17:J17)</f>
         <v/>
       </c>
-      <c r="L17" s="10" t="n"/>
+      <c r="L17" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M17" s="11" t="n"/>
     </row>
     <row r="18">
@@ -1715,7 +1741,9 @@
         <f>SUM(C18:J18)</f>
         <v/>
       </c>
-      <c r="L18" s="10" t="n"/>
+      <c r="L18" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M18" s="11" t="n"/>
     </row>
     <row r="19" ht="15.95" customHeight="1" s="48">
@@ -1753,7 +1781,9 @@
         <f>SUM(C19:J19)</f>
         <v/>
       </c>
-      <c r="L19" s="10" t="n"/>
+      <c r="L19" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M19" s="11" t="n"/>
     </row>
     <row r="20">
@@ -1791,7 +1821,9 @@
         <f>SUM(C20:J20)</f>
         <v/>
       </c>
-      <c r="L20" s="10" t="n"/>
+      <c r="L20" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M20" s="11" t="n"/>
     </row>
     <row r="21" ht="15.95" customHeight="1" s="48">
@@ -1829,7 +1861,9 @@
         <f>SUM(C21:J21)</f>
         <v/>
       </c>
-      <c r="L21" s="10" t="n"/>
+      <c r="L21" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M21" s="11" t="n"/>
     </row>
     <row r="22">
@@ -1867,7 +1901,9 @@
         <f>SUM(C22:J22)</f>
         <v/>
       </c>
-      <c r="L22" s="10" t="n"/>
+      <c r="L22" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M22" s="11" t="n"/>
     </row>
     <row r="23" ht="15.95" customHeight="1" s="48">
@@ -1905,7 +1941,9 @@
         <f>SUM(C23:J23)</f>
         <v/>
       </c>
-      <c r="L23" s="10" t="n"/>
+      <c r="L23" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M23" s="11" t="n"/>
     </row>
     <row r="24">
@@ -1943,7 +1981,9 @@
         <f>SUM(C24:J24)</f>
         <v/>
       </c>
-      <c r="L24" s="10" t="n"/>
+      <c r="L24" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M24" s="11" t="n"/>
     </row>
     <row r="25" ht="15.95" customHeight="1" s="48">
@@ -1981,7 +2021,9 @@
         <f>SUM(C25:J25)</f>
         <v/>
       </c>
-      <c r="L25" s="10" t="n"/>
+      <c r="L25" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M25" s="11" t="n"/>
     </row>
     <row r="26">
@@ -2019,7 +2061,9 @@
         <f>SUM(C26:J26)</f>
         <v/>
       </c>
-      <c r="L26" s="10" t="n"/>
+      <c r="L26" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M26" s="11" t="n"/>
     </row>
     <row r="27" ht="15.95" customHeight="1" s="48">
@@ -2057,7 +2101,9 @@
         <f>SUM(C27:J27)</f>
         <v/>
       </c>
-      <c r="L27" s="10" t="n"/>
+      <c r="L27" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M27" s="11" t="n"/>
     </row>
     <row r="28">
@@ -2095,7 +2141,9 @@
         <f>SUM(C28:J28)</f>
         <v/>
       </c>
-      <c r="L28" s="10" t="n"/>
+      <c r="L28" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M28" s="11" t="n"/>
     </row>
     <row r="29" ht="15.95" customHeight="1" s="48">
@@ -2133,7 +2181,9 @@
         <f>SUM(C29:J29)</f>
         <v/>
       </c>
-      <c r="L29" s="10" t="n"/>
+      <c r="L29" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M29" s="11" t="n"/>
     </row>
     <row r="30">
@@ -2171,7 +2221,9 @@
         <f>SUM(C30:J30)</f>
         <v/>
       </c>
-      <c r="L30" s="10" t="n"/>
+      <c r="L30" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M30" s="11" t="n"/>
     </row>
     <row r="31" ht="15.95" customHeight="1" s="48">
@@ -2209,7 +2261,9 @@
         <f>SUM(C31:J31)</f>
         <v/>
       </c>
-      <c r="L31" s="10" t="n"/>
+      <c r="L31" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M31" s="11" t="n"/>
     </row>
     <row r="32">
@@ -2247,7 +2301,9 @@
         <f>SUM(C32:J32)</f>
         <v/>
       </c>
-      <c r="L32" s="10" t="n"/>
+      <c r="L32" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M32" s="11" t="n"/>
     </row>
     <row r="33" ht="15.95" customHeight="1" s="48">
@@ -2285,7 +2341,9 @@
         <f>SUM(C33:J33)</f>
         <v/>
       </c>
-      <c r="L33" s="10" t="n"/>
+      <c r="L33" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M33" s="11" t="n"/>
     </row>
     <row r="34">
@@ -2323,7 +2381,9 @@
         <f>SUM(C34:J34)</f>
         <v/>
       </c>
-      <c r="L34" s="10" t="n"/>
+      <c r="L34" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M34" s="11" t="n"/>
     </row>
     <row r="35" ht="15.95" customHeight="1" s="48">
@@ -2361,7 +2421,9 @@
         <f>SUM(C35:J35)</f>
         <v/>
       </c>
-      <c r="L35" s="10" t="n"/>
+      <c r="L35" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M35" s="11" t="n"/>
     </row>
     <row r="36">
@@ -2399,7 +2461,9 @@
         <f>SUM(C36:J36)</f>
         <v/>
       </c>
-      <c r="L36" s="10" t="n"/>
+      <c r="L36" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M36" s="11" t="n"/>
     </row>
     <row r="37" ht="15.95" customHeight="1" s="48">
@@ -2437,7 +2501,9 @@
         <f>SUM(C37:J37)</f>
         <v/>
       </c>
-      <c r="L37" s="10" t="n"/>
+      <c r="L37" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M37" s="11" t="n"/>
     </row>
     <row r="38">
@@ -2475,7 +2541,9 @@
         <f>SUM(C38:J38)</f>
         <v/>
       </c>
-      <c r="L38" s="10" t="n"/>
+      <c r="L38" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="M38" s="11" t="n"/>
     </row>
     <row r="39">
@@ -2531,7 +2599,9 @@
         <f>SUM(C40:J40)</f>
         <v/>
       </c>
-      <c r="L40" s="4" t="n"/>
+      <c r="L40" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" ht="15.95" customHeight="1" s="48">
       <c r="A41" s="5" t="n">
@@ -2568,7 +2638,9 @@
         <f>SUM(C41:J41)</f>
         <v/>
       </c>
-      <c r="L41" s="4" t="n"/>
+      <c r="L41" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -2605,7 +2677,9 @@
         <f>SUM(C42:J42)</f>
         <v/>
       </c>
-      <c r="L42" s="4" t="n"/>
+      <c r="L42" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43" ht="15.95" customHeight="1" s="48">
       <c r="A43" s="5" t="n">
@@ -2642,7 +2716,9 @@
         <f>SUM(C43:J43)</f>
         <v/>
       </c>
-      <c r="L43" s="4" t="n"/>
+      <c r="L43" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -2679,7 +2755,9 @@
         <f>SUM(C44:J44)</f>
         <v/>
       </c>
-      <c r="L44" s="4" t="n"/>
+      <c r="L44" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45" ht="15.95" customHeight="1" s="48">
       <c r="A45" s="5" t="n">
@@ -2716,7 +2794,9 @@
         <f>SUM(C45:J45)</f>
         <v/>
       </c>
-      <c r="L45" s="4" t="n"/>
+      <c r="L45" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" ht="15.95" customHeight="1" s="48">
       <c r="A46" s="5" t="n">
@@ -2753,7 +2833,9 @@
         <f>SUM(C46:J46)</f>
         <v/>
       </c>
-      <c r="L46" s="4" t="n"/>
+      <c r="L46" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47" ht="15.95" customHeight="1" s="48">
       <c r="A47" s="5" t="n">
@@ -2790,7 +2872,9 @@
         <f>SUM(C47:J47)</f>
         <v/>
       </c>
-      <c r="L47" s="4" t="n"/>
+      <c r="L47" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48" ht="15.95" customHeight="1" s="48">
       <c r="A48" s="5" t="n">
@@ -2827,7 +2911,9 @@
         <f>SUM(C48:J48)</f>
         <v/>
       </c>
-      <c r="L48" s="4" t="n"/>
+      <c r="L48" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -2864,7 +2950,9 @@
         <f>SUM(C49:J49)</f>
         <v/>
       </c>
-      <c r="L49" s="4" t="n"/>
+      <c r="L49" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50"/>
     <row r="51">
@@ -4665,10 +4753,25 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="54" t="n"/>
-      <c r="C17" s="54" t="n"/>
-      <c r="D17" s="54" t="n"/>
-      <c r="E17" s="55" t="n"/>
+      <c r="B17" s="63" t="inlineStr">
+        <is>
+          <t>Посещаемость по протоколу (за сезон)</t>
+        </is>
+      </c>
+      <c r="C17" s="64">
+        <f>(SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))</f>
+        <v/>
+      </c>
+      <c r="D17" s="63" t="inlineStr">
+        <is>
+          <t>чел.</t>
+        </is>
+      </c>
+      <c r="E17" s="65" t="inlineStr">
+        <is>
+          <t>гр. L — из официального протокола матча</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="63" t="inlineStr">
@@ -4709,10 +4812,25 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="54" t="n"/>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="55" t="n"/>
+      <c r="B20" s="63" t="inlineStr">
+        <is>
+          <t>Отклонение от протокола</t>
+        </is>
+      </c>
+      <c r="C20" s="66">
+        <f>IFERROR((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))/(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)),0)</f>
+        <v/>
+      </c>
+      <c r="D20" s="63" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E20" s="65" t="inlineStr">
+        <is>
+          <t>посещаемость по протоколу / всего билетов</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="63" t="inlineStr">

</xml_diff>

<commit_message>
Tickets: make protocol metric a fact-vs-declared discrepancy
Change the protocol metric from a ratio to the actual discrepancy between
fact (protocol attendance, column L) and the tickets the club declared
(column K): row 20 shows the absolute difference (факт − заявлено, чел.) and
row 26 the relative discrepancy in %. Both are formulas over L and K.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/tickets_calc.xlsx
+++ b/output/tickets_calc.xlsx
@@ -4814,21 +4814,21 @@
     <row r="20">
       <c r="B20" s="63" t="inlineStr">
         <is>
-          <t>Отклонение от протокола</t>
-        </is>
-      </c>
-      <c r="C20" s="66">
-        <f>IFERROR((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))/(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)),0)</f>
+          <t>Расхождение: факт − заявлено (билеты)</t>
+        </is>
+      </c>
+      <c r="C20" s="64">
+        <f>((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))</f>
         <v/>
       </c>
       <c r="D20" s="63" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>чел.</t>
         </is>
       </c>
       <c r="E20" s="65" t="inlineStr">
         <is>
-          <t>посещаемость по протоколу / всего билетов</t>
+          <t>посещаемость по протоколу − всего реализовано билетов</t>
         </is>
       </c>
     </row>
@@ -4918,10 +4918,25 @@
       <c r="E25" s="55" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="54" t="n"/>
-      <c r="C26" s="54" t="n"/>
-      <c r="D26" s="54" t="n"/>
-      <c r="E26" s="55" t="n"/>
+      <c r="B26" s="63" t="inlineStr">
+        <is>
+          <t>Расхождение факта с заявленным, %</t>
+        </is>
+      </c>
+      <c r="C26" s="66">
+        <f>IFERROR(((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))/(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)),0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E26" s="65" t="inlineStr">
+        <is>
+          <t>(протокол − всего билетов) / всего билетов</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="63" t="inlineStr">

</xml_diff>

<commit_message>
Tickets: put protocol attendance in column M (keep Комментарий in L)
In the raw input file column L is «Комментарий» and M is empty, so writing
the protocol column to L overwrote the comments. Move «Посещаемость по
протоколу» to column M (empty) and reference M in the deviation formulas,
leaving «Комментарий» in L intact.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/tickets_calc.xlsx
+++ b/output/tickets_calc.xlsx
@@ -1150,6 +1150,11 @@
       </c>
       <c r="L2" s="44" t="inlineStr">
         <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Посещаемость по протоколу</t>
         </is>
       </c>
@@ -1221,10 +1226,10 @@
         <f>SUM(C5:J5)</f>
         <v/>
       </c>
-      <c r="L5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="11" t="n"/>
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -1261,10 +1266,10 @@
         <f>SUM(C6:J6)</f>
         <v/>
       </c>
-      <c r="L6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="11" t="n"/>
+      <c r="L6" s="10" t="n"/>
+      <c r="M6" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="15.95" customHeight="1" s="48">
       <c r="A7" s="5" t="n">
@@ -1301,10 +1306,10 @@
         <f>SUM(C7:J7)</f>
         <v/>
       </c>
-      <c r="L7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="11" t="n"/>
+      <c r="L7" s="10" t="n"/>
+      <c r="M7" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -1341,10 +1346,10 @@
         <f>SUM(C8:J8)</f>
         <v/>
       </c>
-      <c r="L8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="11" t="n"/>
+      <c r="L8" s="10" t="n"/>
+      <c r="M8" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="15.95" customHeight="1" s="48">
       <c r="A9" s="5" t="n">
@@ -1381,10 +1386,10 @@
         <f>SUM(C9:J9)</f>
         <v/>
       </c>
-      <c r="L9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="11" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="M9" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -1421,10 +1426,10 @@
         <f>SUM(C10:J10)</f>
         <v/>
       </c>
-      <c r="L10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="11" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="M10" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="15.95" customHeight="1" s="48">
       <c r="A11" s="5" t="n">
@@ -1461,10 +1466,10 @@
         <f>SUM(C11:J11)</f>
         <v/>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="11" t="n"/>
+      <c r="L11" s="10" t="n"/>
+      <c r="M11" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1501,10 +1506,10 @@
         <f>SUM(C12:J12)</f>
         <v/>
       </c>
-      <c r="L12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="11" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="15.95" customHeight="1" s="48">
       <c r="A13" s="5" t="n">
@@ -1541,10 +1546,10 @@
         <f>SUM(C13:J13)</f>
         <v/>
       </c>
-      <c r="L13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="11" t="n"/>
+      <c r="L13" s="10" t="n"/>
+      <c r="M13" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1581,10 +1586,10 @@
         <f>SUM(C14:J14)</f>
         <v/>
       </c>
-      <c r="L14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="11" t="n"/>
+      <c r="L14" s="10" t="n"/>
+      <c r="M14" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="15.95" customHeight="1" s="48">
       <c r="A15" s="5" t="n">
@@ -1621,10 +1626,10 @@
         <f>SUM(C15:J15)</f>
         <v/>
       </c>
-      <c r="L15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="11" t="n"/>
+      <c r="L15" s="10" t="n"/>
+      <c r="M15" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1661,10 +1666,10 @@
         <f>SUM(C16:J16)</f>
         <v/>
       </c>
-      <c r="L16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="11" t="n"/>
+      <c r="L16" s="10" t="n"/>
+      <c r="M16" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="15.95" customHeight="1" s="48">
       <c r="A17" s="5" t="n">
@@ -1701,10 +1706,10 @@
         <f>SUM(C17:J17)</f>
         <v/>
       </c>
-      <c r="L17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="11" t="n"/>
+      <c r="L17" s="10" t="n"/>
+      <c r="M17" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1741,10 +1746,10 @@
         <f>SUM(C18:J18)</f>
         <v/>
       </c>
-      <c r="L18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="11" t="n"/>
+      <c r="L18" s="10" t="n"/>
+      <c r="M18" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" ht="15.95" customHeight="1" s="48">
       <c r="A19" s="5" t="n">
@@ -1781,10 +1786,10 @@
         <f>SUM(C19:J19)</f>
         <v/>
       </c>
-      <c r="L19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="11" t="n"/>
+      <c r="L19" s="10" t="n"/>
+      <c r="M19" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1821,10 +1826,10 @@
         <f>SUM(C20:J20)</f>
         <v/>
       </c>
-      <c r="L20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="11" t="n"/>
+      <c r="L20" s="10" t="n"/>
+      <c r="M20" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" ht="15.95" customHeight="1" s="48">
       <c r="A21" s="5" t="n">
@@ -1861,10 +1866,10 @@
         <f>SUM(C21:J21)</f>
         <v/>
       </c>
-      <c r="L21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="11" t="n"/>
+      <c r="L21" s="10" t="n"/>
+      <c r="M21" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1901,10 +1906,10 @@
         <f>SUM(C22:J22)</f>
         <v/>
       </c>
-      <c r="L22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="11" t="n"/>
+      <c r="L22" s="10" t="n"/>
+      <c r="M22" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" ht="15.95" customHeight="1" s="48">
       <c r="A23" s="5" t="n">
@@ -1941,10 +1946,10 @@
         <f>SUM(C23:J23)</f>
         <v/>
       </c>
-      <c r="L23" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="11" t="n"/>
+      <c r="L23" s="10" t="n"/>
+      <c r="M23" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1981,10 +1986,10 @@
         <f>SUM(C24:J24)</f>
         <v/>
       </c>
-      <c r="L24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="11" t="n"/>
+      <c r="L24" s="10" t="n"/>
+      <c r="M24" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="15.95" customHeight="1" s="48">
       <c r="A25" s="5" t="n">
@@ -2021,10 +2026,10 @@
         <f>SUM(C25:J25)</f>
         <v/>
       </c>
-      <c r="L25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="11" t="n"/>
+      <c r="L25" s="10" t="n"/>
+      <c r="M25" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -2061,10 +2066,10 @@
         <f>SUM(C26:J26)</f>
         <v/>
       </c>
-      <c r="L26" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="11" t="n"/>
+      <c r="L26" s="10" t="n"/>
+      <c r="M26" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="15.95" customHeight="1" s="48">
       <c r="A27" s="5" t="n">
@@ -2101,10 +2106,10 @@
         <f>SUM(C27:J27)</f>
         <v/>
       </c>
-      <c r="L27" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="11" t="n"/>
+      <c r="L27" s="10" t="n"/>
+      <c r="M27" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -2141,10 +2146,10 @@
         <f>SUM(C28:J28)</f>
         <v/>
       </c>
-      <c r="L28" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="11" t="n"/>
+      <c r="L28" s="10" t="n"/>
+      <c r="M28" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" ht="15.95" customHeight="1" s="48">
       <c r="A29" s="5" t="n">
@@ -2181,10 +2186,10 @@
         <f>SUM(C29:J29)</f>
         <v/>
       </c>
-      <c r="L29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="11" t="n"/>
+      <c r="L29" s="10" t="n"/>
+      <c r="M29" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -2221,10 +2226,10 @@
         <f>SUM(C30:J30)</f>
         <v/>
       </c>
-      <c r="L30" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="11" t="n"/>
+      <c r="L30" s="10" t="n"/>
+      <c r="M30" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" ht="15.95" customHeight="1" s="48">
       <c r="A31" s="5" t="n">
@@ -2261,10 +2266,10 @@
         <f>SUM(C31:J31)</f>
         <v/>
       </c>
-      <c r="L31" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="11" t="n"/>
+      <c r="L31" s="10" t="n"/>
+      <c r="M31" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -2301,10 +2306,10 @@
         <f>SUM(C32:J32)</f>
         <v/>
       </c>
-      <c r="L32" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="11" t="n"/>
+      <c r="L32" s="10" t="n"/>
+      <c r="M32" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="15.95" customHeight="1" s="48">
       <c r="A33" s="5" t="n">
@@ -2341,10 +2346,10 @@
         <f>SUM(C33:J33)</f>
         <v/>
       </c>
-      <c r="L33" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" s="11" t="n"/>
+      <c r="L33" s="10" t="n"/>
+      <c r="M33" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -2381,10 +2386,10 @@
         <f>SUM(C34:J34)</f>
         <v/>
       </c>
-      <c r="L34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" s="11" t="n"/>
+      <c r="L34" s="10" t="n"/>
+      <c r="M34" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" ht="15.95" customHeight="1" s="48">
       <c r="A35" s="5" t="n">
@@ -2421,10 +2426,10 @@
         <f>SUM(C35:J35)</f>
         <v/>
       </c>
-      <c r="L35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" s="11" t="n"/>
+      <c r="L35" s="10" t="n"/>
+      <c r="M35" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -2461,10 +2466,10 @@
         <f>SUM(C36:J36)</f>
         <v/>
       </c>
-      <c r="L36" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" s="11" t="n"/>
+      <c r="L36" s="10" t="n"/>
+      <c r="M36" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="15.95" customHeight="1" s="48">
       <c r="A37" s="5" t="n">
@@ -2501,10 +2506,10 @@
         <f>SUM(C37:J37)</f>
         <v/>
       </c>
-      <c r="L37" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" s="11" t="n"/>
+      <c r="L37" s="10" t="n"/>
+      <c r="M37" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -2541,10 +2546,10 @@
         <f>SUM(C38:J38)</f>
         <v/>
       </c>
-      <c r="L38" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" s="11" t="n"/>
+      <c r="L38" s="10" t="n"/>
+      <c r="M38" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
@@ -2599,7 +2604,8 @@
         <f>SUM(C40:J40)</f>
         <v/>
       </c>
-      <c r="L40" s="4" t="n">
+      <c r="L40" s="4" t="n"/>
+      <c r="M40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2638,7 +2644,8 @@
         <f>SUM(C41:J41)</f>
         <v/>
       </c>
-      <c r="L41" s="4" t="n">
+      <c r="L41" s="4" t="n"/>
+      <c r="M41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2677,7 +2684,8 @@
         <f>SUM(C42:J42)</f>
         <v/>
       </c>
-      <c r="L42" s="4" t="n">
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2716,7 +2724,8 @@
         <f>SUM(C43:J43)</f>
         <v/>
       </c>
-      <c r="L43" s="4" t="n">
+      <c r="L43" s="4" t="n"/>
+      <c r="M43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2755,7 +2764,8 @@
         <f>SUM(C44:J44)</f>
         <v/>
       </c>
-      <c r="L44" s="4" t="n">
+      <c r="L44" s="4" t="n"/>
+      <c r="M44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2794,7 +2804,8 @@
         <f>SUM(C45:J45)</f>
         <v/>
       </c>
-      <c r="L45" s="4" t="n">
+      <c r="L45" s="4" t="n"/>
+      <c r="M45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2833,7 +2844,8 @@
         <f>SUM(C46:J46)</f>
         <v/>
       </c>
-      <c r="L46" s="4" t="n">
+      <c r="L46" s="4" t="n"/>
+      <c r="M46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2872,7 +2884,8 @@
         <f>SUM(C47:J47)</f>
         <v/>
       </c>
-      <c r="L47" s="4" t="n">
+      <c r="L47" s="4" t="n"/>
+      <c r="M47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2911,7 +2924,8 @@
         <f>SUM(C48:J48)</f>
         <v/>
       </c>
-      <c r="L48" s="4" t="n">
+      <c r="L48" s="4" t="n"/>
+      <c r="M48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2950,7 +2964,8 @@
         <f>SUM(C49:J49)</f>
         <v/>
       </c>
-      <c r="L49" s="4" t="n">
+      <c r="L49" s="4" t="n"/>
+      <c r="M49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4759,7 +4774,7 @@
         </is>
       </c>
       <c r="C17" s="64">
-        <f>(SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))</f>
+        <f>(SUM('Реализованные билеты'!M5:M38)+SUM('Реализованные билеты'!M40:M49))</f>
         <v/>
       </c>
       <c r="D17" s="63" t="inlineStr">
@@ -4769,7 +4784,7 @@
       </c>
       <c r="E17" s="65" t="inlineStr">
         <is>
-          <t>гр. L — из официального протокола матча</t>
+          <t>гр. M — из официального протокола матча</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4833,7 @@
         </is>
       </c>
       <c r="C20" s="64">
-        <f>((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))</f>
+        <f>((SUM('Реализованные билеты'!M5:M38)+SUM('Реализованные билеты'!M40:M49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))</f>
         <v/>
       </c>
       <c r="D20" s="63" t="inlineStr">
@@ -4924,7 +4939,7 @@
         </is>
       </c>
       <c r="C26" s="66">
-        <f>IFERROR(((SUM('Реализованные билеты'!L5:L38)+SUM('Реализованные билеты'!L40:L49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))/(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)),0)</f>
+        <f>IFERROR(((SUM('Реализованные билеты'!M5:M38)+SUM('Реализованные билеты'!M40:M49))-(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)))/(SUM('Реализованные билеты'!K5:K38)+SUM('Реализованные билеты'!K40:K49)),0)</f>
         <v/>
       </c>
       <c r="D26" s="63" t="inlineStr">

</xml_diff>

<commit_message>
Tickets: default agent commission to a number for calculations
The «Размер агентской комиссии, %» field arrives as text (« - »), so the
commission metric returned "нет данных". Convert the placeholder in the
agent table's commission column to numeric 0, and point the C52 formula at
the actual first-agent row (previously it hit the merged-header row) with a
VALUE() fallback for numeric-text. Commission now computes (0% by default).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/tickets_calc.xlsx
+++ b/output/tickets_calc.xlsx
@@ -4313,10 +4313,8 @@
           <t xml:space="preserve"> - </t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - </t>
-        </is>
+      <c r="D4" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
@@ -5384,7 +5382,7 @@
         </is>
       </c>
       <c r="C52" s="66">
-        <f>IF(ISNUMBER('Агенты и онлайн продажи'!D3),'Агенты и онлайн продажи'!D3/100,"нет данных")</f>
+        <f>IF(ISNUMBER('Агенты и онлайн продажи'!D4),'Агенты и онлайн продажи'!D4/100,IFERROR(VALUE('Агенты и онлайн продажи'!D4)/100,0))</f>
         <v/>
       </c>
       <c r="D52" s="63" t="inlineStr">
@@ -5392,7 +5390,11 @@
           <t>%</t>
         </is>
       </c>
-      <c r="E52" s="55" t="n"/>
+      <c r="E52" s="65" t="inlineStr">
+        <is>
+          <t>по умолчанию 0; заполняется в таблице агентов</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="54" t="n"/>

</xml_diff>

<commit_message>
Tickets: agent commission = average across agents, not a single cell
Change «Агентская комиссия» to AVERAGE over the commission column across all
agent rows (÷100), wrapped in IFERROR→0 for an empty table. AVERAGE ignores
text placeholders (« - ») and blanks, so the metric reflects the mean of real
agent commissions. No longer forces the placeholder cell to 0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/tickets_calc.xlsx
+++ b/output/tickets_calc.xlsx
@@ -4313,8 +4313,10 @@
           <t xml:space="preserve"> - </t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
-        <v>0</v>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - </t>
+        </is>
       </c>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
@@ -5378,11 +5380,11 @@
     <row r="52">
       <c r="B52" s="63" t="inlineStr">
         <is>
-          <t>Агентская комиссия</t>
+          <t>Агентская комиссия (средняя по агентам)</t>
         </is>
       </c>
       <c r="C52" s="66">
-        <f>IF(ISNUMBER('Агенты и онлайн продажи'!D4),'Агенты и онлайн продажи'!D4/100,IFERROR(VALUE('Агенты и онлайн продажи'!D4)/100,0))</f>
+        <f>IFERROR(AVERAGE('Агенты и онлайн продажи'!D4:D7)/100,0)</f>
         <v/>
       </c>
       <c r="D52" s="63" t="inlineStr">
@@ -5392,7 +5394,7 @@
       </c>
       <c r="E52" s="65" t="inlineStr">
         <is>
-          <t>по умолчанию 0; заполняется в таблице агентов</t>
+          <t>среднее по столбцу комиссии; пустые/« - » не учитываются</t>
         </is>
       </c>
     </row>

</xml_diff>